<commit_message>
Add WK1ST/WK2ND suffix to booking and stock-balance block headers
BOOKING (BKK/LCH) and STOCK BALANCE END WK (BKK/LCH) headers in rows 29
(WK1ST) and 43 (WK2ND) now carry their week slot, e.g.
'BOOKING (BKK) WK1ST'. Re-built 2026-10-05 with it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-5/Stock Daily 2026-10-05.xlsx
+++ b/10-5/Stock Daily 2026-10-05.xlsx
@@ -4000,7 +4000,7 @@
       <c r="B29" s="186" t="n"/>
       <c r="C29" s="151" t="inlineStr">
         <is>
-          <t>BOOKING (BKK)</t>
+          <t>BOOKING (BKK) WK1ST</t>
         </is>
       </c>
       <c r="D29" s="187" t="n"/>
@@ -4017,7 +4017,7 @@
       <c r="K29" s="190" t="n"/>
       <c r="L29" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (BKK)</t>
+          <t>STOCK BALANCE END WK (BKK) WK1ST</t>
         </is>
       </c>
       <c r="M29" s="187" t="n"/>
@@ -4037,7 +4037,7 @@
       <c r="W29" s="186" t="n"/>
       <c r="X29" s="151" t="inlineStr">
         <is>
-          <t>BOOKING (LCH)</t>
+          <t>BOOKING (LCH) WK1ST</t>
         </is>
       </c>
       <c r="Y29" s="187" t="n"/>
@@ -4054,7 +4054,7 @@
       <c r="AF29" s="190" t="n"/>
       <c r="AG29" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (LCH)</t>
+          <t>STOCK BALANCE END WK (LCH) WK1ST</t>
         </is>
       </c>
       <c r="AH29" s="187" t="n"/>
@@ -5536,7 +5536,7 @@
       <c r="B43" s="186" t="n"/>
       <c r="C43" s="151" t="inlineStr">
         <is>
-          <t>BOOKING (BKK)</t>
+          <t>BOOKING (BKK) WK2ND</t>
         </is>
       </c>
       <c r="D43" s="187" t="n"/>
@@ -5553,7 +5553,7 @@
       <c r="K43" s="190" t="n"/>
       <c r="L43" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (BKK)</t>
+          <t>STOCK BALANCE END WK (BKK) WK2ND</t>
         </is>
       </c>
       <c r="M43" s="187" t="n"/>
@@ -5573,7 +5573,7 @@
       <c r="W43" s="186" t="n"/>
       <c r="X43" s="151" t="inlineStr">
         <is>
-          <t>BOOKING (LCH)</t>
+          <t>BOOKING (LCH) WK2ND</t>
         </is>
       </c>
       <c r="Y43" s="187" t="n"/>
@@ -5590,7 +5590,7 @@
       <c r="AF43" s="190" t="n"/>
       <c r="AG43" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (LCH)</t>
+          <t>STOCK BALANCE END WK (LCH) WK2ND</t>
         </is>
       </c>
       <c r="AH43" s="187" t="n"/>

</xml_diff>

<commit_message>
Blank STOCK BALANCE END WK (LCH) cells for LCMT/ESCO/LCIT/HPT
Per sirichai: the four LCH terminal groups show no empty-container
balance in the WK1ST and WK2ND blocks. Formulas removed from those
cells (so the block TOTAL excludes them too); CURRENT STOCK, FULL INBOUND
and BOOKING rows for them are unchanged. Re-built 2026-10-05.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-5/Stock Daily 2026-10-05.xlsx
+++ b/10-5/Stock Daily 2026-10-05.xlsx
@@ -4332,42 +4332,15 @@
       <c r="AD31" s="229" t="n"/>
       <c r="AE31" s="229" t="n"/>
       <c r="AF31" s="230" t="n"/>
-      <c r="AG31" s="225">
-        <f>SUM(AG4-X31)</f>
-        <v/>
-      </c>
-      <c r="AH31" s="226">
-        <f>SUM(AH4-Y31)</f>
-        <v/>
-      </c>
-      <c r="AI31" s="226">
-        <f>SUM(AI4-Z31)</f>
-        <v/>
-      </c>
-      <c r="AJ31" s="226">
-        <f>SUM(AJ4-AA31)</f>
-        <v/>
-      </c>
-      <c r="AK31" s="226">
-        <f>SUM(AK4-AB31)</f>
-        <v/>
-      </c>
-      <c r="AL31" s="226">
-        <f>SUM(AL4-AC31)</f>
-        <v/>
-      </c>
-      <c r="AM31" s="226">
-        <f>SUM(AM4-AD31)</f>
-        <v/>
-      </c>
-      <c r="AN31" s="226">
-        <f>SUM(AN4-AE31)</f>
-        <v/>
-      </c>
-      <c r="AO31" s="227">
-        <f>SUM(AO4-AF31)</f>
-        <v/>
-      </c>
+      <c r="AG31" s="225" t="n"/>
+      <c r="AH31" s="226" t="n"/>
+      <c r="AI31" s="226" t="n"/>
+      <c r="AJ31" s="226" t="n"/>
+      <c r="AK31" s="226" t="n"/>
+      <c r="AL31" s="226" t="n"/>
+      <c r="AM31" s="226" t="n"/>
+      <c r="AN31" s="226" t="n"/>
+      <c r="AO31" s="227" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="43" t="inlineStr">
@@ -4448,42 +4421,15 @@
       <c r="AD32" s="235" t="n"/>
       <c r="AE32" s="235" t="n"/>
       <c r="AF32" s="236" t="n"/>
-      <c r="AG32" s="231">
-        <f>SUM(AG5-X32)</f>
-        <v/>
-      </c>
-      <c r="AH32" s="232">
-        <f>SUM(AH5-Y32)</f>
-        <v/>
-      </c>
-      <c r="AI32" s="232">
-        <f>SUM(AI5-Z32)</f>
-        <v/>
-      </c>
-      <c r="AJ32" s="232">
-        <f>SUM(AJ5-AA32)</f>
-        <v/>
-      </c>
-      <c r="AK32" s="232">
-        <f>SUM(AK5-AB32)</f>
-        <v/>
-      </c>
-      <c r="AL32" s="232">
-        <f>SUM(AL5-AC32)</f>
-        <v/>
-      </c>
-      <c r="AM32" s="232">
-        <f>SUM(AM5-AD32)</f>
-        <v/>
-      </c>
-      <c r="AN32" s="232">
-        <f>SUM(AN5-AE32)</f>
-        <v/>
-      </c>
-      <c r="AO32" s="233">
-        <f>SUM(AO5-AF32)</f>
-        <v/>
-      </c>
+      <c r="AG32" s="231" t="n"/>
+      <c r="AH32" s="232" t="n"/>
+      <c r="AI32" s="232" t="n"/>
+      <c r="AJ32" s="232" t="n"/>
+      <c r="AK32" s="232" t="n"/>
+      <c r="AL32" s="232" t="n"/>
+      <c r="AM32" s="232" t="n"/>
+      <c r="AN32" s="232" t="n"/>
+      <c r="AO32" s="233" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
@@ -4560,42 +4506,15 @@
       <c r="AD33" s="235" t="n"/>
       <c r="AE33" s="235" t="n"/>
       <c r="AF33" s="236" t="n"/>
-      <c r="AG33" s="231">
-        <f>SUM(AG6-X33)</f>
-        <v/>
-      </c>
-      <c r="AH33" s="232">
-        <f>SUM(AH6-Y33)</f>
-        <v/>
-      </c>
-      <c r="AI33" s="232">
-        <f>SUM(AI6-Z33)</f>
-        <v/>
-      </c>
-      <c r="AJ33" s="232">
-        <f>SUM(AJ6-AA33)</f>
-        <v/>
-      </c>
-      <c r="AK33" s="232">
-        <f>SUM(AK6-AB33)</f>
-        <v/>
-      </c>
-      <c r="AL33" s="232">
-        <f>SUM(AL6-AC33)</f>
-        <v/>
-      </c>
-      <c r="AM33" s="232">
-        <f>SUM(AM6-AD33)</f>
-        <v/>
-      </c>
-      <c r="AN33" s="232">
-        <f>SUM(AN6-AE33)</f>
-        <v/>
-      </c>
-      <c r="AO33" s="233">
-        <f>SUM(AO6-AF33)</f>
-        <v/>
-      </c>
+      <c r="AG33" s="231" t="n"/>
+      <c r="AH33" s="232" t="n"/>
+      <c r="AI33" s="232" t="n"/>
+      <c r="AJ33" s="232" t="n"/>
+      <c r="AK33" s="232" t="n"/>
+      <c r="AL33" s="232" t="n"/>
+      <c r="AM33" s="232" t="n"/>
+      <c r="AN33" s="232" t="n"/>
+      <c r="AO33" s="233" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="136" t="inlineStr">
@@ -4672,42 +4591,15 @@
       <c r="AD34" s="235" t="n"/>
       <c r="AE34" s="235" t="n"/>
       <c r="AF34" s="236" t="n"/>
-      <c r="AG34" s="231">
-        <f>SUM(AG7-X34)</f>
-        <v/>
-      </c>
-      <c r="AH34" s="232">
-        <f>SUM(AH7-Y34)</f>
-        <v/>
-      </c>
-      <c r="AI34" s="232">
-        <f>SUM(AI7-Z34)</f>
-        <v/>
-      </c>
-      <c r="AJ34" s="232">
-        <f>SUM(AJ7-AA34)</f>
-        <v/>
-      </c>
-      <c r="AK34" s="232">
-        <f>SUM(AK7-AB34)</f>
-        <v/>
-      </c>
-      <c r="AL34" s="232">
-        <f>SUM(AL7-AC34)</f>
-        <v/>
-      </c>
-      <c r="AM34" s="232">
-        <f>SUM(AM7-AD34)</f>
-        <v/>
-      </c>
-      <c r="AN34" s="232">
-        <f>SUM(AN7-AE34)</f>
-        <v/>
-      </c>
-      <c r="AO34" s="233">
-        <f>SUM(AO7-AF34)</f>
-        <v/>
-      </c>
+      <c r="AG34" s="231" t="n"/>
+      <c r="AH34" s="232" t="n"/>
+      <c r="AI34" s="232" t="n"/>
+      <c r="AJ34" s="232" t="n"/>
+      <c r="AK34" s="232" t="n"/>
+      <c r="AL34" s="232" t="n"/>
+      <c r="AM34" s="232" t="n"/>
+      <c r="AN34" s="232" t="n"/>
+      <c r="AO34" s="233" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="43" t="inlineStr">
@@ -5868,42 +5760,15 @@
       <c r="AD45" s="229" t="n"/>
       <c r="AE45" s="229" t="n"/>
       <c r="AF45" s="230" t="n"/>
-      <c r="AG45" s="225">
-        <f>SUM(AG31-X45)</f>
-        <v/>
-      </c>
-      <c r="AH45" s="226">
-        <f>SUM(AH31-Y45)</f>
-        <v/>
-      </c>
-      <c r="AI45" s="226">
-        <f>SUM(AI31-Z45)</f>
-        <v/>
-      </c>
-      <c r="AJ45" s="226">
-        <f>SUM(AJ31-AA45)</f>
-        <v/>
-      </c>
-      <c r="AK45" s="226">
-        <f>SUM(AK31-AB45)</f>
-        <v/>
-      </c>
-      <c r="AL45" s="226">
-        <f>SUM(AL31-AC45)</f>
-        <v/>
-      </c>
-      <c r="AM45" s="226">
-        <f>SUM(AM31-AD45)</f>
-        <v/>
-      </c>
-      <c r="AN45" s="226">
-        <f>SUM(AN31-AE45)</f>
-        <v/>
-      </c>
-      <c r="AO45" s="227">
-        <f>SUM(AO31-AF45)</f>
-        <v/>
-      </c>
+      <c r="AG45" s="225" t="n"/>
+      <c r="AH45" s="226" t="n"/>
+      <c r="AI45" s="226" t="n"/>
+      <c r="AJ45" s="226" t="n"/>
+      <c r="AK45" s="226" t="n"/>
+      <c r="AL45" s="226" t="n"/>
+      <c r="AM45" s="226" t="n"/>
+      <c r="AN45" s="226" t="n"/>
+      <c r="AO45" s="227" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="43" t="inlineStr">
@@ -5984,42 +5849,15 @@
       <c r="AD46" s="235" t="n"/>
       <c r="AE46" s="235" t="n"/>
       <c r="AF46" s="236" t="n"/>
-      <c r="AG46" s="231">
-        <f>SUM(AG32-X46)</f>
-        <v/>
-      </c>
-      <c r="AH46" s="232">
-        <f>SUM(AH32-Y46)</f>
-        <v/>
-      </c>
-      <c r="AI46" s="232">
-        <f>SUM(AI32-Z46)</f>
-        <v/>
-      </c>
-      <c r="AJ46" s="232">
-        <f>SUM(AJ32-AA46)</f>
-        <v/>
-      </c>
-      <c r="AK46" s="232">
-        <f>SUM(AK32-AB46)</f>
-        <v/>
-      </c>
-      <c r="AL46" s="232">
-        <f>SUM(AL32-AC46)</f>
-        <v/>
-      </c>
-      <c r="AM46" s="232">
-        <f>SUM(AM32-AD46)</f>
-        <v/>
-      </c>
-      <c r="AN46" s="232">
-        <f>SUM(AN32-AE46)</f>
-        <v/>
-      </c>
-      <c r="AO46" s="233">
-        <f>SUM(AO32-AF46)</f>
-        <v/>
-      </c>
+      <c r="AG46" s="231" t="n"/>
+      <c r="AH46" s="232" t="n"/>
+      <c r="AI46" s="232" t="n"/>
+      <c r="AJ46" s="232" t="n"/>
+      <c r="AK46" s="232" t="n"/>
+      <c r="AL46" s="232" t="n"/>
+      <c r="AM46" s="232" t="n"/>
+      <c r="AN46" s="232" t="n"/>
+      <c r="AO46" s="233" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="23" t="inlineStr">
@@ -6096,42 +5934,15 @@
       <c r="AD47" s="235" t="n"/>
       <c r="AE47" s="235" t="n"/>
       <c r="AF47" s="236" t="n"/>
-      <c r="AG47" s="231">
-        <f>SUM(AG33-X47)</f>
-        <v/>
-      </c>
-      <c r="AH47" s="232">
-        <f>SUM(AH33-Y47)</f>
-        <v/>
-      </c>
-      <c r="AI47" s="232">
-        <f>SUM(AI33-Z47)</f>
-        <v/>
-      </c>
-      <c r="AJ47" s="232">
-        <f>SUM(AJ33-AA47)</f>
-        <v/>
-      </c>
-      <c r="AK47" s="232">
-        <f>SUM(AK33-AB47)</f>
-        <v/>
-      </c>
-      <c r="AL47" s="232">
-        <f>SUM(AL33-AC47)</f>
-        <v/>
-      </c>
-      <c r="AM47" s="232">
-        <f>SUM(AM33-AD47)</f>
-        <v/>
-      </c>
-      <c r="AN47" s="232">
-        <f>SUM(AN33-AE47)</f>
-        <v/>
-      </c>
-      <c r="AO47" s="233">
-        <f>SUM(AO33-AF47)</f>
-        <v/>
-      </c>
+      <c r="AG47" s="231" t="n"/>
+      <c r="AH47" s="232" t="n"/>
+      <c r="AI47" s="232" t="n"/>
+      <c r="AJ47" s="232" t="n"/>
+      <c r="AK47" s="232" t="n"/>
+      <c r="AL47" s="232" t="n"/>
+      <c r="AM47" s="232" t="n"/>
+      <c r="AN47" s="232" t="n"/>
+      <c r="AO47" s="233" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="136" t="inlineStr">
@@ -6208,42 +6019,15 @@
       <c r="AD48" s="235" t="n"/>
       <c r="AE48" s="235" t="n"/>
       <c r="AF48" s="236" t="n"/>
-      <c r="AG48" s="231">
-        <f>SUM(AG34-X48)</f>
-        <v/>
-      </c>
-      <c r="AH48" s="232">
-        <f>SUM(AH34-Y48)</f>
-        <v/>
-      </c>
-      <c r="AI48" s="232">
-        <f>SUM(AI34-Z48)</f>
-        <v/>
-      </c>
-      <c r="AJ48" s="232">
-        <f>SUM(AJ34-AA48)</f>
-        <v/>
-      </c>
-      <c r="AK48" s="232">
-        <f>SUM(AK34-AB48)</f>
-        <v/>
-      </c>
-      <c r="AL48" s="232">
-        <f>SUM(AL34-AC48)</f>
-        <v/>
-      </c>
-      <c r="AM48" s="232">
-        <f>SUM(AM34-AD48)</f>
-        <v/>
-      </c>
-      <c r="AN48" s="232">
-        <f>SUM(AN34-AE48)</f>
-        <v/>
-      </c>
-      <c r="AO48" s="233">
-        <f>SUM(AO34-AF48)</f>
-        <v/>
-      </c>
+      <c r="AG48" s="231" t="n"/>
+      <c r="AH48" s="232" t="n"/>
+      <c r="AI48" s="232" t="n"/>
+      <c r="AJ48" s="232" t="n"/>
+      <c r="AK48" s="232" t="n"/>
+      <c r="AL48" s="232" t="n"/>
+      <c r="AM48" s="232" t="n"/>
+      <c r="AN48" s="232" t="n"/>
+      <c r="AO48" s="233" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="43" t="inlineStr">

</xml_diff>

<commit_message>
Rename block headers: STOCK BALANCE END WK (X) -> STOCK BALANCE END (X)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-5/Stock Daily 2026-10-05.xlsx
+++ b/10-5/Stock Daily 2026-10-05.xlsx
@@ -4017,7 +4017,7 @@
       <c r="K29" s="190" t="n"/>
       <c r="L29" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (BKK) WK1ST</t>
+          <t>STOCK BALANCE END (BKK) WK1ST</t>
         </is>
       </c>
       <c r="M29" s="187" t="n"/>
@@ -4054,7 +4054,7 @@
       <c r="AF29" s="190" t="n"/>
       <c r="AG29" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (LCH) WK1ST</t>
+          <t>STOCK BALANCE END (LCH) WK1ST</t>
         </is>
       </c>
       <c r="AH29" s="187" t="n"/>
@@ -5445,7 +5445,7 @@
       <c r="K43" s="190" t="n"/>
       <c r="L43" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (BKK) WK2ND</t>
+          <t>STOCK BALANCE END (BKK) WK2ND</t>
         </is>
       </c>
       <c r="M43" s="187" t="n"/>
@@ -5482,7 +5482,7 @@
       <c r="AF43" s="190" t="n"/>
       <c r="AG43" s="143" t="inlineStr">
         <is>
-          <t>STOCK BALANCE END WK (LCH) WK2ND</t>
+          <t>STOCK BALANCE END (LCH) WK2ND</t>
         </is>
       </c>
       <c r="AH43" s="187" t="n"/>

</xml_diff>